<commit_message>
feat: close Phase C commercial data solidity
Ship Neon audit/documents, tenant export and Blob backup crons, supplier/event import, and multi-user revision conflict polling so the core is sellable without data-loss risk.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/assets/lean-event/import/lean-event-rubrica-sedi.xlsx
+++ b/public/assets/lean-event/import/lean-event-rubrica-sedi.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A6"/>
   <cols>
     <col min="1" max="1" width="72.83203125" customWidth="1"/>
   </cols>
@@ -430,27 +430,12 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>URL scheda esterna: link opzionale (es. MeetingeCongressi).</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>URL immagine: copertina sede (link diretto a JPG/PNG/WebP).</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Salva come .xlsx e carica quando disponibile l'import sedi.</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
         <v>Formati accettati: .xlsx, .csv (separatore ; o ,)</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A6"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>